<commit_message>
First ML version, with code, pretrain data and sensor, nozzle data and surrogate
</commit_message>
<xml_diff>
--- a/plug_result_mesh.xlsx
+++ b/plug_result_mesh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nozzle\OpenFOAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{309F3AF7-420E-49B6-993C-4C28A79AE697}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B65929-50D9-4CA6-9B27-1AB08275908F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24165" windowHeight="11415" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,11 +25,11 @@
     <sheet name="150" sheetId="5" r:id="rId10"/>
     <sheet name="100" sheetId="6" r:id="rId11"/>
     <sheet name="50" sheetId="9" r:id="rId12"/>
-    <sheet name="对比" sheetId="14" r:id="rId13"/>
-    <sheet name="分析（150）" sheetId="15" r:id="rId14"/>
+    <sheet name="compare" sheetId="16" r:id="rId13"/>
+    <sheet name="对比" sheetId="14" r:id="rId14"/>
+    <sheet name="分析（150）" sheetId="15" r:id="rId15"/>
   </sheets>
   <calcPr calcId="179021"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -9758,6 +9758,142 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ECC837B-4BAA-4C79-8C51-D4C09F81E16F}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1">
+        <v>150</v>
+      </c>
+      <c r="B1">
+        <v>300</v>
+      </c>
+      <c r="C1">
+        <v>600</v>
+      </c>
+      <c r="D1">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1.83136151283953</v>
+      </c>
+      <c r="B2">
+        <v>1.8193998285838</v>
+      </c>
+      <c r="C2">
+        <v>1.8133733600045601</v>
+      </c>
+      <c r="D2">
+        <v>1.8118409309843699</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>1.8190907148078399</v>
+      </c>
+      <c r="B3">
+        <v>1.8100950426148901</v>
+      </c>
+      <c r="C3">
+        <v>1.80542058611956</v>
+      </c>
+      <c r="D3">
+        <v>1.80058941622812</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>1.81691227391257</v>
+      </c>
+      <c r="B4">
+        <v>1.8006356868417499</v>
+      </c>
+      <c r="C4">
+        <v>1.7951875993439099</v>
+      </c>
+      <c r="D4">
+        <v>1.79255673827282</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>1.7981498911257401</v>
+      </c>
+      <c r="B5">
+        <v>1.7873000397107801</v>
+      </c>
+      <c r="C5">
+        <v>1.78272702353042</v>
+      </c>
+      <c r="D5">
+        <v>1.78079830545315</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>1.77744676236324</v>
+      </c>
+      <c r="B6">
+        <v>1.76720093208658</v>
+      </c>
+      <c r="C6">
+        <v>1.7619508527769701</v>
+      </c>
+      <c r="D6">
+        <v>1.76113845685016</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>1.7424455784408399</v>
+      </c>
+      <c r="B7">
+        <v>1.7338508308896099</v>
+      </c>
+      <c r="C7">
+        <v>1.7291884580469901</v>
+      </c>
+      <c r="D7">
+        <v>1.7281815291795699</v>
+      </c>
+      <c r="E7" s="1"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <conditionalFormatting sqref="E2:E7">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color theme="0"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color theme="0"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF9B32DC-EDDC-4214-8F2E-13B059234E89}">
   <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
@@ -10378,7 +10514,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD52A78D-FEBE-4DBB-B5EE-5D3BABD670C5}">
   <dimension ref="A1:AA26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>

</xml_diff>